<commit_message>
split code into modules and formatted
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -472,10 +472,10 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>79261</v>
+        <v>79783</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1587639613393</v>
+        <v>1597744779814</v>
       </c>
     </row>
     <row r="3">
@@ -493,10 +493,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2252.95</v>
+        <v>2266.04</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>271904664118</v>
+        <v>273398692827</v>
       </c>
     </row>
     <row r="4">
@@ -514,10 +514,10 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.99953</v>
+        <v>0.999474</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>189727282890</v>
+        <v>189758461996</v>
       </c>
     </row>
     <row r="5">
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>669.6799999999999</v>
+        <v>672.65</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>90255562721</v>
+        <v>90639556938</v>
       </c>
     </row>
     <row r="6">
@@ -556,10 +556,10 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.42</v>
+        <v>1.43</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>87801432654</v>
+        <v>88593502326</v>
       </c>
     </row>
     <row r="7">
@@ -577,10 +577,10 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1</v>
+        <v>0.999684</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>76761744262</v>
+        <v>76706290771</v>
       </c>
     </row>
     <row r="8">
@@ -598,10 +598,10 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>91.06999999999999</v>
+        <v>91.05</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>52640683503</v>
+        <v>52617662963</v>
       </c>
     </row>
     <row r="9">
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.349579</v>
+        <v>0.351777</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>33140458127</v>
+        <v>33346015223</v>
       </c>
     </row>
     <row r="10">
@@ -640,10 +640,10 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1.044</v>
+        <v>1.034</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>18479987175</v>
+        <v>18300558754</v>
       </c>
     </row>
     <row r="11">
@@ -661,10 +661,10 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.112748</v>
+        <v>0.113329</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>17388970573</v>
+        <v>17468051524</v>
       </c>
     </row>
     <row r="12">
@@ -682,10 +682,10 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>58.3</v>
+        <v>58.68</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>12404094191</v>
+        <v>12490654454</v>
       </c>
     </row>
     <row r="13">
@@ -703,10 +703,10 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.999674</v>
+        <v>0.999673</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>10995747218</v>
+        <v>10984936011</v>
       </c>
     </row>
     <row r="14">
@@ -724,10 +724,10 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.263556</v>
+        <v>0.264981</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>9748508101</v>
+        <v>9798825709</v>
       </c>
     </row>
     <row r="15">
@@ -736,19 +736,19 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hyperliquid</t>
+          <t>LEO Token</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>hype</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>38.89</v>
+        <v>10.13</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>9264964416</v>
+        <v>9331252532</v>
       </c>
     </row>
     <row r="16">
@@ -757,19 +757,19 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>LEO Token</t>
+          <t>Hyperliquid</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>hype</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>10.06</v>
+        <v>38.99</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>9260561596</v>
+        <v>9296206740</v>
       </c>
     </row>
     <row r="17">
@@ -787,10 +787,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>521.97</v>
+        <v>521.37</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>8711189168</v>
+        <v>8710782126</v>
       </c>
     </row>
     <row r="18">
@@ -808,10 +808,10 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>433.27</v>
+        <v>433.61</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>8679978026</v>
+        <v>8688044510</v>
       </c>
     </row>
     <row r="19">
@@ -829,10 +829,10 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>10.16</v>
+        <v>10.27</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>7387375504</v>
+        <v>7462246877</v>
       </c>
     </row>
     <row r="20">
@@ -850,10 +850,10 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>393.03</v>
+        <v>394.9</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>7249213598</v>
+        <v>7283999237</v>
       </c>
     </row>
     <row r="21">
@@ -871,10 +871,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.154229</v>
+        <v>0.158083</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>5937105211</v>
+        <v>6089737331</v>
       </c>
     </row>
     <row r="22">
@@ -892,10 +892,10 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>2.1</v>
+        <v>2.12</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>5624903158</v>
+        <v>5709127682</v>
       </c>
     </row>
     <row r="23">
@@ -913,10 +913,10 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.158735</v>
+        <v>0.159268</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>5315204177</v>
+        <v>5333662927</v>
       </c>
     </row>
     <row r="24">
@@ -937,7 +937,7 @@
         <v>1.2</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>4798933375</v>
+        <v>4796513553</v>
       </c>
     </row>
     <row r="25">
@@ -955,10 +955,10 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.999236</v>
+        <v>0.999231</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>4418461573</v>
+        <v>4432471731</v>
       </c>
     </row>
     <row r="26">
@@ -967,19 +967,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dai</t>
+          <t>Litecoin</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>dai</t>
+          <t>ltc</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.999595</v>
+        <v>57.11</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>4379551018</v>
+        <v>4407895421</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added fixes and formatted modules
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -472,10 +472,10 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>79783</v>
+        <v>79573</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1597744779814</v>
+        <v>1594422071836</v>
       </c>
     </row>
     <row r="3">
@@ -493,10 +493,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2266.04</v>
+        <v>2253.03</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>273398692827</v>
+        <v>272100075792</v>
       </c>
     </row>
     <row r="4">
@@ -514,10 +514,10 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.999474</v>
+        <v>0.999497</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>189758461996</v>
+        <v>189762789418</v>
       </c>
     </row>
     <row r="5">
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>672.65</v>
+        <v>669.5700000000001</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>90639556938</v>
+        <v>90292503624</v>
       </c>
     </row>
     <row r="6">
@@ -559,7 +559,7 @@
         <v>1.43</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>88593502326</v>
+        <v>88248457963</v>
       </c>
     </row>
     <row r="7">
@@ -577,10 +577,10 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.999684</v>
+        <v>0.9996119999999999</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>76706290771</v>
+        <v>76711644182</v>
       </c>
     </row>
     <row r="8">
@@ -598,10 +598,10 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>91.05</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>52617662963</v>
+        <v>52365657811</v>
       </c>
     </row>
     <row r="9">
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.351777</v>
+        <v>0.35271</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>33346015223</v>
+        <v>33432447853</v>
       </c>
     </row>
     <row r="10">
@@ -661,10 +661,10 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.113329</v>
+        <v>0.112887</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>17468051524</v>
+        <v>17421535739</v>
       </c>
     </row>
     <row r="12">
@@ -682,10 +682,10 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>58.68</v>
+        <v>58.58</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>12490654454</v>
+        <v>12479088135</v>
       </c>
     </row>
     <row r="13">
@@ -703,10 +703,10 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.999673</v>
+        <v>0.999689</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>10984936011</v>
+        <v>10983637991</v>
       </c>
     </row>
     <row r="14">
@@ -724,10 +724,10 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.264981</v>
+        <v>0.263835</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>9798825709</v>
+        <v>9764187806</v>
       </c>
     </row>
     <row r="15">
@@ -745,10 +745,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>10.13</v>
+        <v>10.17</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>9331252532</v>
+        <v>9362136861</v>
       </c>
     </row>
     <row r="16">
@@ -766,10 +766,10 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>38.99</v>
+        <v>38.92</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>9296206740</v>
+        <v>9295864879</v>
       </c>
     </row>
     <row r="17">
@@ -787,10 +787,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>521.37</v>
+        <v>522.99</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>8710782126</v>
+        <v>8741564015</v>
       </c>
     </row>
     <row r="18">
@@ -808,10 +808,10 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>433.61</v>
+        <v>433.12</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>8688044510</v>
+        <v>8677370954</v>
       </c>
     </row>
     <row r="19">
@@ -829,10 +829,10 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>10.27</v>
+        <v>10.19</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>7462246877</v>
+        <v>7414362943</v>
       </c>
     </row>
     <row r="20">
@@ -850,10 +850,10 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>394.9</v>
+        <v>394.3</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>7283999237</v>
+        <v>7274620700</v>
       </c>
     </row>
     <row r="21">
@@ -871,10 +871,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.158083</v>
+        <v>0.157998</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>6089737331</v>
+        <v>6062116404</v>
       </c>
     </row>
     <row r="22">
@@ -892,10 +892,10 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>2.12</v>
+        <v>2.11</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>5709127682</v>
+        <v>5673189630</v>
       </c>
     </row>
     <row r="23">
@@ -913,10 +913,10 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.159268</v>
+        <v>0.158436</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>5333662927</v>
+        <v>5307079316</v>
       </c>
     </row>
     <row r="24">
@@ -934,10 +934,10 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>1.2</v>
+        <v>1.19</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>4796513553</v>
+        <v>4786882310</v>
       </c>
     </row>
     <row r="25">
@@ -955,10 +955,10 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.999231</v>
+        <v>0.999541</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>4432471731</v>
+        <v>4432221013</v>
       </c>
     </row>
     <row r="26">
@@ -976,10 +976,10 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>57.11</v>
+        <v>56.9</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>4407895421</v>
+        <v>4391953286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>